<commit_message>
feat: implement WordReaderHelper for .docx parsing and add standard exam import templates
</commit_message>
<xml_diff>
--- a/templates/exam_import_template_annotated.xlsx
+++ b/templates/exam_import_template_annotated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\examination\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{234024F5-4C81-4098-A14A-2FE78AE619EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80B065C3-2EB5-462D-870D-DCF1F62DC116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,9 @@
     <t>จงยกตัวอย่างองค์ประกอบพื้นฐานของคอมพิวเตอร์ (Hardware) มาอย่างน้อย 3 ประการ</t>
   </si>
   <si>
-    <t>1. หน่วยประมวลผลกลาง (CPU) 2. หน่วยความจำหลัก (RAM) 3. อุปกรณ์จัดเก็บข้อมูล (Hard Disk / SSD)</t>
+    <t>1. หน่วยประมวลผลกลาง (CPU) 
+2. หน่วยความจำหลัก (RAM) 
+3. อุปกรณ์จัดเก็บข้อมูล (Hard Disk / SSD)</t>
   </si>
 </sst>
 </file>
@@ -542,8 +544,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - ส่วนที่ถูกเน้น1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -944,14 +949,14 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="207" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>